<commit_message>
R04: correções da revisão adversarial e relatório final
- motor: o piso de viabilidade redistribui a partir do VBP inicial em cada
  iteração (sem catraca quando o piso baixa); pesos_tust_geracao exige uma
  linha por região e subsetor de geração e o roteamento por componentes
- TUST do SOL-RS/PET-RS latentes marcada como hipótese (coef_latentes e
  relatório); alternativa do SOL com a TUST/MWh do RS na aba B_TWh
- fontes do GAS-RB em componentes_v03 (principal e _gas4dist); ressalva
  sobre PIS/Cofins do SEAMSE; LEIAME das simulações; figuras refeitas
- relatório RODADA_04_resposta.md completo, HISTORICO, README e LEIAME
- 2 testes novos; 389 testes passam

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/parametros/quadro_parametros_v03.xlsx
+++ b/parametros/quadro_parametros_v03.xlsx
@@ -2860,7 +2860,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>D9-b (variante): preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
+          <t>V2 (Rodada 04): principal — preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>D9-b: preço médio das 4 distribuidoras (cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16; nan) × volume não térmico (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
+          <t>V2 (Rodada 04): sensibilidade _gas4dist — preço médio das 4 distribuidoras (o principal da v02) (cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16) × volume não térmico (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D9-b (variante): preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
+          <t>V2 (Rodada 04): principal — preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D9-b: preço médio das 4 distribuidoras (cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16; nan) × volume não térmico (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
+          <t>V2 (Rodada 04): sensibilidade _gas4dist — preço médio das 4 distribuidoras (o principal da v02) (cálculo do projeto com as DFP 2019 de Sulgás, Comgás, CEG e Gasmig, ver linhas sulgas_*, comgas_*, ceg_*, gasmig_* (Σ receita líquida de venda de gás não térmica (14738.052 R$ mi) ÷ Σ volume não térmico (7627.178 milhões m³)); acesso 2026-10-16) × volume não térmico (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5453,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D9-b (variante): preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
+          <t>V2 (Rodada 04): principal — preço da Sulgás 2019 (1.390413 R$/m³; Sulgás (demonstrações contábeis publicadas pela CAGE/Sefaz-RS), Prestação de Contas do Governador 2019, Volume V parte 2 (Setor Empresarial), Demonstrações Contábeis da Sulgás 2019, DRE (PDF p. 69, 'Receita líquida - venda de gás e serviços' (Nota 17), 31/12/2019 = 898.710.338,54; repetido na Nota 18 (p. 86)); acesso 2026-10-15T19:34:32Z; https://cage.fazenda.rs.gov.br/upload/arquivos/202507/02143858-prestacao-de-contas-do-governador-2019-v-5-2.pdf) × volume não térmico do RB (MME (fonte da tabela: Abegás), Boletim Mensal de Acompanhamento da Indústria de Gás Natural nº 154 (dez/2019) (p. 16, 'Demanda de Gás Natural por Distribuidora (sem o segmento termelétrico)', linha 'TOTAL DISTRIBUIDORAS SEM O SEGMENTO TERMELÉTRICO', 'Média 2019'); acesso 2026-10-15T19:36:10Z; https://www.gov.br/mme/pt-br/assuntos/secretarias/petroleo-gas-natural-e-biocombustiveis/publicacoes-1/boletim-mensal-de-acompanhamento-da-industria-de-gas-natural/2019/12-boletim-mensal-de-acompanhamento-da-industria-de-gas-natural-dezembro-2019.pdf)</t>
         </is>
       </c>
     </row>

</xml_diff>